<commit_message>
mensagem de alteração/inclusão ajustada
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -277,11 +277,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3990,14 +3990,14 @@
     <col width="20.453125" customWidth="1" style="29" min="6" max="6"/>
     <col width="8.1796875" customWidth="1" style="29" min="7" max="7"/>
     <col width="8" customWidth="1" style="29" min="8" max="9"/>
-    <col width="9.1796875" customWidth="1" style="29" min="10" max="17"/>
-    <col width="9.1796875" customWidth="1" style="29" min="18" max="16384"/>
+    <col width="9.1796875" customWidth="1" style="29" min="10" max="18"/>
+    <col width="9.1796875" customWidth="1" style="29" min="19" max="16384"/>
   </cols>
   <sheetData>
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Transmissores de Pressão Diferencial</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO FORTE</t>
+          <t>FPSO Forte</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>FIT-1231010T-DPT</t>
+          <t>FIT-1231006-PT</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Gás Importado</t>
+          <t>Export Gas</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25 - ODS - 70 - PRE - 494</t>
+          <t>25-ODS-70 - PRE - 373</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4081,9 +4081,9 @@
           <t>Data de Calibração:</t>
         </is>
       </c>
-      <c r="C9" s="27" t="inlineStr">
-        <is>
-          <t>14/11/2025</t>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>25/08/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>29/08/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4613,7 +4613,7 @@
     <row r="41" ht="36" customHeight="1">
       <c r="B41" s="9" t="n"/>
       <c r="C41" s="10" t="n"/>
-      <c r="D41" s="26" t="inlineStr">
+      <c r="D41" s="27" t="inlineStr">
         <is>
           <t>Responsável pela análise</t>
         </is>

</xml_diff>

<commit_message>
ajuste interface range indicado TE
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -3990,14 +3990,14 @@
     <col width="20.453125" customWidth="1" style="29" min="6" max="6"/>
     <col width="8.1796875" customWidth="1" style="29" min="7" max="7"/>
     <col width="8" customWidth="1" style="29" min="8" max="9"/>
-    <col width="9.1796875" customWidth="1" style="29" min="10" max="18"/>
-    <col width="9.1796875" customWidth="1" style="29" min="19" max="16384"/>
+    <col width="9.1796875" customWidth="1" style="29" min="10" max="20"/>
+    <col width="9.1796875" customWidth="1" style="29" min="21" max="16384"/>
   </cols>
   <sheetData>
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Transmissores de Pressão</t>
+          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO Forte</t>
+          <t>FPSO-FRADE</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>FIT-1231006-PT</t>
+          <t>044-TE-1020A</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Export Gas</t>
+          <t>Oil to Cargo A</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-70 - PRE - 373</t>
+          <t>25-ODS-37 - TEM - 504</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>25/08/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>29/08/2025</t>
+          <t>23/12/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
ajuste XML para armazenamento do cert. TE no TT
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>044-TE-1020A</t>
+          <t>044-TT-1020A</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37 - TEM - 504</t>
+          <t>25-ODS-37 - TEM - 505</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>

</xml_diff>

<commit_message>
ajust final da inclusão do certificado do tt no Te
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO-FRADE</t>
+          <t>FPSO Forte</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>044-TT-1020A</t>
+          <t>FIT-1231006-TT</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Oil to Cargo A</t>
+          <t>Export Gas</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37 - TEM - 505</t>
+          <t>25-ODS-37 - TEM - 302</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>25/08/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>23/12/2025</t>
+          <t>29/08/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
tratativa xml pressao diferencial - FPSO BRAVO (regra exclusiva
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -3997,7 +3997,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão Diferencial</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO Forte</t>
+          <t>FPSO FORTE</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>FIT-1231006-TT</t>
+          <t>FIT-1231010T-DPT</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Export Gas</t>
+          <t>Gás Importado</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37 - TEM - 302</t>
+          <t>25 - ODS - 70 - PRE - 494</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>25/08/2025</t>
+          <t>14/11/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>29/08/2025</t>
+          <t>17/11/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
ajuste de descrição visor de resultados
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -3997,7 +3997,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Transmissores de Pressão Diferencial</t>
+          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO FORTE</t>
+          <t>FPSO-FRADE</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>FIT-1231010T-DPT</t>
+          <t>044-TT-1020A</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Gás Importado</t>
+          <t>Oil to Cargo A</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25 - ODS - 70 - PRE - 494</t>
+          <t>25-ODS-37 - TEM - 505</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>14/11/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>23/12/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
atualização de funcionalidades readme
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO-FRADE</t>
+          <t>FPSO FORTE</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>044-TT-1020A</t>
+          <t>FIT-1231010A-TT</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Oil to Cargo A</t>
+          <t>Gás Lift A- Poço ABL-81</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37 - TEM - 505</t>
+          <t>25 - ODS - 70 - TEM - 456</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>22/11/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>23/12/2025</t>
+          <t>25/11/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4637,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="C9:D9"/>
-    <mergeCell ref="D41:E41"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
ajuste na geração do xml
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO FORTE</t>
+          <t>FPSO-FRADE</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>FIT-1231010A-TT</t>
+          <t>044-TT-1020A</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Gás Lift A- Poço ABL-81</t>
+          <t>Oil to Cargo A</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25 - ODS - 70 - TEM - 456</t>
+          <t>25-ODS-37 - TEM - 505</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>22/11/2025</t>
+          <t>21/12/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>25/11/2025</t>
+          <t>23/12/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>

</xml_diff>

<commit_message>
regra mvs alterada para qualquer contrato
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -3997,7 +3997,7 @@
     <row r="2" ht="37.5" customHeight="1">
       <c r="B2" s="34" t="inlineStr">
         <is>
-          <t>Análise Crítica de Calibração dos Sensores de Temperatura</t>
+          <t>Análise Crítica de Calibração dos Transmissores de Pressão Diferencial</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO-FRADE</t>
+          <t>ORIGEM ENERGIA ALAGOAS S.A.</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>044-TT-1020A</t>
+          <t>PDT-SG-122104-01</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4055,11 +4055,7 @@
           <t>Localização:</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>Oil to Cargo A</t>
-        </is>
-      </c>
+      <c r="C8" s="18" t="n"/>
       <c r="D8" s="20" t="n"/>
       <c r="E8" s="6" t="inlineStr">
         <is>
@@ -4068,7 +4064,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25-ODS-37 - TEM - 505</t>
+          <t>25-ODS-0638 - PRE - 231</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4079,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>21/12/2025</t>
+          <t>01/09/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4601,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>23/12/2025</t>
+          <t>15/09/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>
@@ -4637,9 +4633,9 @@
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B39:I39"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="C9:D9"/>
     <mergeCell ref="D41:E41"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B4:I5"/>

</xml_diff>

<commit_message>
CMC instrumentos de pressão sem conversão 5
</commit_message>
<xml_diff>
--- a/TemplateAC.xlsx
+++ b/TemplateAC.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="15420" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="17565" yWindow="-11370" windowWidth="21600" windowHeight="11175" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="BASE" sheetId="1" state="hidden" r:id="rId1"/>
@@ -3990,8 +3990,8 @@
     <col width="20.453125" customWidth="1" style="29" min="6" max="6"/>
     <col width="8.1796875" customWidth="1" style="29" min="7" max="7"/>
     <col width="8" customWidth="1" style="29" min="8" max="9"/>
-    <col width="9.1796875" customWidth="1" style="29" min="10" max="20"/>
-    <col width="9.1796875" customWidth="1" style="29" min="21" max="16384"/>
+    <col width="9.1796875" customWidth="1" style="29" min="10" max="21"/>
+    <col width="9.1796875" customWidth="1" style="29" min="22" max="16384"/>
   </cols>
   <sheetData>
     <row r="2" ht="37.5" customHeight="1">
@@ -4031,7 +4031,7 @@
       </c>
       <c r="C7" s="35" t="inlineStr">
         <is>
-          <t>FPSO FORTE</t>
+          <t>FPSO BRAVO</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>FIT-1231010A-TT</t>
+          <t>TIT-1198A-62</t>
         </is>
       </c>
       <c r="G7" s="19" t="n"/>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Gás Lift A- Poço ABL-81</t>
+          <t>Processo para Tanque de Carga - Tramo C</t>
         </is>
       </c>
       <c r="D8" s="20" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>25 - ODS - 70 - TEM - 456</t>
+          <t>25-ODS-53 - TEM - 472</t>
         </is>
       </c>
       <c r="G8" s="19" t="n"/>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t>22/11/2025</t>
+          <t>24/11/2025</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -4605,7 +4605,7 @@
       <c r="G40" s="15" t="n"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>25/11/2025</t>
+          <t>28/11/2025</t>
         </is>
       </c>
       <c r="I40" s="16" t="n"/>

</xml_diff>